<commit_message>
Adding simulation based on changes of LPC
</commit_message>
<xml_diff>
--- a/SType2.xlsx
+++ b/SType2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_LASSO\LAS_Simulation_Jateng\I-O_Analysis\Regional-Economy---Jawa-Tengah\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7BF3532E-FAB5-48B3-A691-CEF810CCACA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC004F7D-703C-4BE4-AAA7-0B26F71BC891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E5C01E36-476D-4251-853A-101B82F37DF2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E5C01E36-476D-4251-853A-101B82F37DF2}"/>
   </bookViews>
   <sheets>
     <sheet name="SType2" sheetId="1" r:id="rId1"/>
@@ -39,212 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
-  <si>
-    <t>KodeSektor</t>
-  </si>
-  <si>
-    <t>NamaSektor</t>
-  </si>
-  <si>
-    <t>Padi</t>
-  </si>
-  <si>
-    <t>Jagung</t>
-  </si>
-  <si>
-    <t>Tanaman pangan dan tanaman semusim lainnya</t>
-  </si>
-  <si>
-    <t>Hortikultura, tanaman hias, dan pengembangbiakan tanaman</t>
-  </si>
-  <si>
-    <t>Tebu</t>
-  </si>
-  <si>
-    <t>Tembakau</t>
-  </si>
-  <si>
-    <t>Kelapa dan tanaman penghasil minyak lainnya</t>
-  </si>
-  <si>
-    <t>Kopi, teh, dan kakao</t>
-  </si>
-  <si>
-    <t>Rempah, tanaman aromatik, dan tanaman obat</t>
-  </si>
-  <si>
-    <t>Karet dan tanaman tahunan lainnya</t>
-  </si>
-  <si>
-    <t>Peternakan dan hasil-hasilnya</t>
-  </si>
-  <si>
-    <t>Jasa pertanian, pascapanen, perburuan, dan kegiatan penunjang</t>
-  </si>
-  <si>
-    <t>Kehutanan dan penebangan kayu</t>
-  </si>
-  <si>
-    <t>Perikanan tangkap</t>
-  </si>
-  <si>
-    <t>Perikanan budidaya</t>
-  </si>
-  <si>
-    <t>Minyak bumi, gas bumi, panas bumi, dan jasa penunjangnya</t>
-  </si>
-  <si>
-    <t>Batubara, bijih logam, mineral lainnya, dan jasa penunjang</t>
-  </si>
-  <si>
-    <t>Penggalian batu, pasir, tanah liat, garam, dan penggalian lainnya</t>
-  </si>
-  <si>
-    <t>Industri produk batubara dan pengilangan minyak bumi</t>
-  </si>
-  <si>
-    <t>Industri pengolahan daging, ikan, buah, dan sayuran</t>
-  </si>
-  <si>
-    <t>Industri minyak, lemak, dan produk susu</t>
-  </si>
-  <si>
-    <t>Industri penggilingan padi-padian, tepung, dan pati</t>
-  </si>
-  <si>
-    <t>Industri gula</t>
-  </si>
-  <si>
-    <t>Industri roti, mi, cokelat, kopi/teh olahan, bumbu, dan makanan lainnya</t>
-  </si>
-  <si>
-    <t>Industri makanan hewan atau pakan</t>
-  </si>
-  <si>
-    <t>Industri minuman</t>
-  </si>
-  <si>
-    <t>Industri pengolahan tembakau</t>
-  </si>
-  <si>
-    <t>Industri tekstil</t>
-  </si>
-  <si>
-    <t>Industri pakaian jadi</t>
-  </si>
-  <si>
-    <t>Industri kulit, barang dari kulit, dan alas kaki</t>
-  </si>
-  <si>
-    <t>Industri kayu, barang dari kayu, bambu, rotan, dan sejenisnya</t>
-  </si>
-  <si>
-    <t>Industri kertas, barang dari kertas, pencetakan, dan reproduksi media</t>
-  </si>
-  <si>
-    <t>Industri kimia, farmasi, dan obat tradisional</t>
-  </si>
-  <si>
-    <t>Industri karet, barang dari karet, dan plastik</t>
-  </si>
-  <si>
-    <t>Industri barang galian bukan logam</t>
-  </si>
-  <si>
-    <t>Industri logam dasar</t>
-  </si>
-  <si>
-    <t>Industri barang logam, bukan mesin dan peralatannya</t>
-  </si>
-  <si>
-    <t>Industri barang logam, komputer, elektronik, optik, dan peralatan listrik</t>
-  </si>
-  <si>
-    <t>Industri mesin dan perlengkapan</t>
-  </si>
-  <si>
-    <t>Industri kendaraan bermotor dan alat angkutan lainnya</t>
-  </si>
-  <si>
-    <t>Industri furnitur</t>
-  </si>
-  <si>
-    <t>Industri pengolahan lainnya serta reparasi dan pemasangan mesin</t>
-  </si>
-  <si>
-    <t>Ketenagalistrikan</t>
-  </si>
-  <si>
-    <t>Pengadaan gas, uap/air panas, udara dingin, dan produksi es</t>
-  </si>
-  <si>
-    <t>Pengadaan air; pengelolaan sampah, limbah, dan daur ulang</t>
-  </si>
-  <si>
-    <t>Konstruksi</t>
-  </si>
-  <si>
-    <t>Perdagangan, reparasi dan perawatan mobil dan sepeda motor</t>
-  </si>
-  <si>
-    <t>Perdagangan besar dan eceran, bukan mobil dan sepeda motor</t>
-  </si>
-  <si>
-    <t>Angkutan darat, rel, dan angkutan melalui saluran pipa</t>
-  </si>
-  <si>
-    <t>Angkutan udara</t>
-  </si>
-  <si>
-    <t>Angkutan perairan</t>
-  </si>
-  <si>
-    <t>Pergudangan dan aktivitas penunjang angkutan</t>
-  </si>
-  <si>
-    <t>Aktivitas pos dan kurir</t>
-  </si>
-  <si>
-    <t>Penyediaan akomodasi</t>
-  </si>
-  <si>
-    <t>Penyediaan makanan dan minuman</t>
-  </si>
-  <si>
-    <t>Informasi dan komunikasi</t>
-  </si>
-  <si>
-    <t>Aktivitas jasa keuangan, bukan asuransi dan dana pensiun</t>
-  </si>
-  <si>
-    <t>Asuransi, penjaminan, reasuransi, dan dana pensiun</t>
-  </si>
-  <si>
-    <t>Aktivitas penunjang jasa keuangan dan asuransi</t>
-  </si>
-  <si>
-    <t>Real estat</t>
-  </si>
-  <si>
-    <t>Jasa profesional, ilmiah, teknis, penyewaan, ketenagakerjaan, dan penunjang usaha</t>
-  </si>
-  <si>
-    <t>Administrasi pemerintahan, pertahanan, dan jaminan sosial wajib</t>
-  </si>
-  <si>
-    <t>Pendidikan</t>
-  </si>
-  <si>
-    <t>Kesehatan manusia dan kegiatan sosial</t>
-  </si>
-  <si>
-    <t>Jasa lainnya, kesenian, rumah tangga pemberi kerja, dan badan internasional</t>
-  </si>
-  <si>
-    <t>Sektor ekonomi lain yang tidak jelas batasannya</t>
-  </si>
-</sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -457,90 +252,80 @@
   <sheetPr>
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:W67"/>
+  <dimension ref="A1:U66"/>
   <sheetFormatPr defaultRowHeight="14"/>
-  <cols>
-    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="70.25" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:23">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="1" spans="1:21">
+      <c r="A1">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0</v>
       </c>
       <c r="C1">
-        <v>2025</v>
+        <v>0</v>
       </c>
       <c r="D1">
-        <v>2026</v>
+        <v>0</v>
       </c>
       <c r="E1">
-        <v>2027</v>
+        <v>0</v>
       </c>
       <c r="F1">
-        <v>2028</v>
+        <v>0</v>
       </c>
       <c r="G1">
-        <v>2029</v>
+        <v>0</v>
       </c>
       <c r="H1">
-        <v>2030</v>
+        <v>0</v>
       </c>
       <c r="I1">
-        <v>2031</v>
+        <v>0</v>
       </c>
       <c r="J1">
-        <v>2032</v>
+        <v>0</v>
       </c>
       <c r="K1">
-        <v>2033</v>
+        <v>0</v>
       </c>
       <c r="L1">
-        <v>2034</v>
+        <v>0</v>
       </c>
       <c r="M1">
-        <v>2035</v>
+        <v>0</v>
       </c>
       <c r="N1">
-        <v>2036</v>
+        <v>0</v>
       </c>
       <c r="O1">
-        <v>2037</v>
+        <v>0</v>
       </c>
       <c r="P1">
-        <v>2038</v>
+        <v>0</v>
       </c>
       <c r="Q1">
-        <v>2039</v>
+        <v>0</v>
       </c>
       <c r="R1">
-        <v>2040</v>
+        <v>0</v>
       </c>
       <c r="S1">
-        <v>2041</v>
+        <v>0</v>
       </c>
       <c r="T1">
-        <v>2042</v>
+        <v>0</v>
       </c>
       <c r="U1">
-        <v>2043</v>
-      </c>
-      <c r="V1">
-        <v>2044</v>
-      </c>
-      <c r="W1">
-        <v>2045</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21">
       <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -549,69 +334,63 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="Q2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="S2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="T2">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21">
       <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -620,10 +399,10 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G3">
         <v>0.01</v>
@@ -632,10 +411,10 @@
         <v>0.01</v>
       </c>
       <c r="I3">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="J3">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K3">
         <v>0.03</v>
@@ -644,45 +423,39 @@
         <v>0.03</v>
       </c>
       <c r="M3">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="N3">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="O3">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="P3">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="Q3">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="R3">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="S3">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="T3">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="U3">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="V3">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="W3">
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21">
       <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -691,10 +464,10 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G4">
         <v>0.01</v>
@@ -703,10 +476,10 @@
         <v>0.01</v>
       </c>
       <c r="I4">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="J4">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K4">
         <v>0.03</v>
@@ -715,10 +488,10 @@
         <v>0.03</v>
       </c>
       <c r="M4">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="N4">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="O4">
         <v>0.05</v>
@@ -741,244 +514,220 @@
       <c r="U4">
         <v>0.05</v>
       </c>
-      <c r="V4">
+    </row>
+    <row r="5" spans="1:21">
+      <c r="A5">
+        <v>0</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21">
+      <c r="A6">
+        <v>0</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0.01</v>
+      </c>
+      <c r="F7">
+        <v>0.01</v>
+      </c>
+      <c r="G7">
+        <v>0.01</v>
+      </c>
+      <c r="H7">
+        <v>0.01</v>
+      </c>
+      <c r="I7">
+        <v>0.03</v>
+      </c>
+      <c r="J7">
+        <v>0.03</v>
+      </c>
+      <c r="K7">
+        <v>0.03</v>
+      </c>
+      <c r="L7">
+        <v>0.03</v>
+      </c>
+      <c r="M7">
         <v>0.05</v>
       </c>
-      <c r="W4">
+      <c r="N7">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="5" spans="1:23">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
+      <c r="O7">
+        <v>0.05</v>
+      </c>
+      <c r="P7">
+        <v>0.05</v>
+      </c>
+      <c r="Q7">
+        <v>0.05</v>
+      </c>
+      <c r="R7">
+        <v>0.05</v>
+      </c>
+      <c r="S7">
+        <v>0.05</v>
+      </c>
+      <c r="T7">
+        <v>0.05</v>
+      </c>
+      <c r="U7">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21">
+      <c r="A8">
+        <v>0</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
         <v>0.01</v>
       </c>
-      <c r="H5">
+      <c r="F8">
         <v>0.01</v>
-      </c>
-      <c r="I5">
-        <v>0.01</v>
-      </c>
-      <c r="J5">
-        <v>0.01</v>
-      </c>
-      <c r="K5">
-        <v>0.03</v>
-      </c>
-      <c r="L5">
-        <v>0.03</v>
-      </c>
-      <c r="M5">
-        <v>0.03</v>
-      </c>
-      <c r="N5">
-        <v>0.03</v>
-      </c>
-      <c r="O5">
-        <v>0.05</v>
-      </c>
-      <c r="P5">
-        <v>0.05</v>
-      </c>
-      <c r="Q5">
-        <v>0.05</v>
-      </c>
-      <c r="R5">
-        <v>0.05</v>
-      </c>
-      <c r="S5">
-        <v>0.05</v>
-      </c>
-      <c r="T5">
-        <v>0.05</v>
-      </c>
-      <c r="U5">
-        <v>0.05</v>
-      </c>
-      <c r="V5">
-        <v>0.05</v>
-      </c>
-      <c r="W5">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-      <c r="T6">
-        <v>0</v>
-      </c>
-      <c r="U6">
-        <v>0</v>
-      </c>
-      <c r="V6">
-        <v>0</v>
-      </c>
-      <c r="W6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>0</v>
-      </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
-      <c r="T7">
-        <v>0</v>
-      </c>
-      <c r="U7">
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <v>0</v>
-      </c>
-      <c r="W7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
       </c>
       <c r="G8">
         <v>0.01</v>
@@ -987,10 +736,10 @@
         <v>0.01</v>
       </c>
       <c r="I8">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="J8">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="K8">
         <v>0.03</v>
@@ -999,10 +748,10 @@
         <v>0.03</v>
       </c>
       <c r="M8">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="N8">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="O8">
         <v>0.05</v>
@@ -1025,516 +774,468 @@
       <c r="U8">
         <v>0.05</v>
       </c>
-      <c r="V8">
+    </row>
+    <row r="9" spans="1:21">
+      <c r="A9">
+        <v>0</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21">
+      <c r="A10">
+        <v>0</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0.01</v>
+      </c>
+      <c r="F10">
+        <v>0.01</v>
+      </c>
+      <c r="G10">
+        <v>0.01</v>
+      </c>
+      <c r="H10">
+        <v>0.01</v>
+      </c>
+      <c r="I10">
+        <v>0.03</v>
+      </c>
+      <c r="J10">
+        <v>0.03</v>
+      </c>
+      <c r="K10">
+        <v>0.03</v>
+      </c>
+      <c r="L10">
+        <v>0.03</v>
+      </c>
+      <c r="M10">
         <v>0.05</v>
       </c>
-      <c r="W8">
+      <c r="N10">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="9" spans="1:23">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
+      <c r="O10">
+        <v>0.05</v>
+      </c>
+      <c r="P10">
+        <v>0.05</v>
+      </c>
+      <c r="Q10">
+        <v>0.05</v>
+      </c>
+      <c r="R10">
+        <v>0.05</v>
+      </c>
+      <c r="S10">
+        <v>0.05</v>
+      </c>
+      <c r="T10">
+        <v>0.05</v>
+      </c>
+      <c r="U10">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21">
+      <c r="A11">
+        <v>0</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21">
+      <c r="A12">
+        <v>0</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21">
+      <c r="A13">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21">
+      <c r="A14">
+        <v>0</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21">
+      <c r="A15">
+        <v>0</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
         <v>0.01</v>
       </c>
-      <c r="H9">
+      <c r="F15">
         <v>0.01</v>
       </c>
-      <c r="I9">
+      <c r="G15">
         <v>0.01</v>
       </c>
-      <c r="J9">
+      <c r="H15">
         <v>0.01</v>
       </c>
-      <c r="K9">
+      <c r="I15">
         <v>0.03</v>
       </c>
-      <c r="L9">
+      <c r="J15">
         <v>0.03</v>
       </c>
-      <c r="M9">
+      <c r="K15">
         <v>0.03</v>
       </c>
-      <c r="N9">
+      <c r="L15">
         <v>0.03</v>
       </c>
-      <c r="O9">
-        <v>0.05</v>
-      </c>
-      <c r="P9">
-        <v>0.05</v>
-      </c>
-      <c r="Q9">
-        <v>0.05</v>
-      </c>
-      <c r="R9">
-        <v>0.05</v>
-      </c>
-      <c r="S9">
-        <v>0.05</v>
-      </c>
-      <c r="T9">
-        <v>0.05</v>
-      </c>
-      <c r="U9">
-        <v>0.05</v>
-      </c>
-      <c r="V9">
-        <v>0.05</v>
-      </c>
-      <c r="W9">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
-      </c>
-      <c r="Q10">
-        <v>0</v>
-      </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
-      <c r="T10">
-        <v>0</v>
-      </c>
-      <c r="U10">
-        <v>0</v>
-      </c>
-      <c r="V10">
-        <v>0</v>
-      </c>
-      <c r="W10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>0.01</v>
-      </c>
-      <c r="H11">
-        <v>0.01</v>
-      </c>
-      <c r="I11">
-        <v>0.01</v>
-      </c>
-      <c r="J11">
-        <v>0.01</v>
-      </c>
-      <c r="K11">
-        <v>0.03</v>
-      </c>
-      <c r="L11">
-        <v>0.03</v>
-      </c>
-      <c r="M11">
-        <v>0.03</v>
-      </c>
-      <c r="N11">
-        <v>0.03</v>
-      </c>
-      <c r="O11">
-        <v>0.05</v>
-      </c>
-      <c r="P11">
-        <v>0.05</v>
-      </c>
-      <c r="Q11">
-        <v>0.05</v>
-      </c>
-      <c r="R11">
-        <v>0.05</v>
-      </c>
-      <c r="S11">
-        <v>0.05</v>
-      </c>
-      <c r="T11">
-        <v>0.05</v>
-      </c>
-      <c r="U11">
-        <v>0.05</v>
-      </c>
-      <c r="V11">
-        <v>0.05</v>
-      </c>
-      <c r="W11">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-      <c r="I12">
-        <v>0</v>
-      </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>0</v>
-      </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="P12">
-        <v>0</v>
-      </c>
-      <c r="Q12">
-        <v>0</v>
-      </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12">
-        <v>0</v>
-      </c>
-      <c r="T12">
-        <v>0</v>
-      </c>
-      <c r="U12">
-        <v>0</v>
-      </c>
-      <c r="V12">
-        <v>0</v>
-      </c>
-      <c r="W12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
-      <c r="N13">
-        <v>0</v>
-      </c>
-      <c r="O13">
-        <v>0</v>
-      </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
-      <c r="Q13">
-        <v>0</v>
-      </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13">
-        <v>0</v>
-      </c>
-      <c r="T13">
-        <v>0</v>
-      </c>
-      <c r="U13">
-        <v>0</v>
-      </c>
-      <c r="V13">
-        <v>0</v>
-      </c>
-      <c r="W13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14">
-        <v>0</v>
-      </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-      <c r="N14">
-        <v>0</v>
-      </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
-        <v>0</v>
-      </c>
-      <c r="Q14">
-        <v>0</v>
-      </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <v>0</v>
-      </c>
-      <c r="T14">
-        <v>0</v>
-      </c>
-      <c r="U14">
-        <v>0</v>
-      </c>
-      <c r="V14">
-        <v>0</v>
-      </c>
-      <c r="W14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
-        <v>0</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
       <c r="M15">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="N15">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="P15">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="Q15">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="R15">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="S15">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="T15">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="U15">
-        <v>0</v>
-      </c>
-      <c r="V15">
-        <v>0</v>
-      </c>
-      <c r="W15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21">
       <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>16</v>
+        <v>0</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1549,63 +1250,57 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="J16">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="K16">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="L16">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="M16">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="N16">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="O16">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="P16">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="Q16">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="R16">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="S16">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="T16">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="U16">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="V16">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="W16">
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21">
       <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>17</v>
+        <v>0</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1664,19 +1359,13 @@
       <c r="U17">
         <v>0</v>
       </c>
-      <c r="V17">
-        <v>0</v>
-      </c>
-      <c r="W17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23">
+    </row>
+    <row r="18" spans="1:21">
       <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>18</v>
+        <v>0</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1735,19 +1424,13 @@
       <c r="U18">
         <v>0</v>
       </c>
-      <c r="V18">
-        <v>0</v>
-      </c>
-      <c r="W18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23">
+    </row>
+    <row r="19" spans="1:21">
       <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1806,19 +1489,13 @@
       <c r="U19">
         <v>0</v>
       </c>
-      <c r="V19">
-        <v>0</v>
-      </c>
-      <c r="W19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23">
+    </row>
+    <row r="20" spans="1:21">
       <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>20</v>
+        <v>0</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1877,19 +1554,13 @@
       <c r="U20">
         <v>0</v>
       </c>
-      <c r="V20">
-        <v>0</v>
-      </c>
-      <c r="W20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23">
+    </row>
+    <row r="21" spans="1:21">
       <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>21</v>
+        <v>0</v>
+      </c>
+      <c r="B21">
+        <v>0</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1948,19 +1619,13 @@
       <c r="U21">
         <v>0</v>
       </c>
-      <c r="V21">
-        <v>0</v>
-      </c>
-      <c r="W21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:23">
+    </row>
+    <row r="22" spans="1:21">
       <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>22</v>
+        <v>0</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -2019,19 +1684,13 @@
       <c r="U22">
         <v>0</v>
       </c>
-      <c r="V22">
-        <v>0</v>
-      </c>
-      <c r="W22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:23">
+    </row>
+    <row r="23" spans="1:21">
       <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>23</v>
+        <v>0</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2090,19 +1749,13 @@
       <c r="U23">
         <v>0</v>
       </c>
-      <c r="V23">
-        <v>0</v>
-      </c>
-      <c r="W23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23">
+    </row>
+    <row r="24" spans="1:21">
       <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>24</v>
+        <v>0</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -2161,19 +1814,13 @@
       <c r="U24">
         <v>0</v>
       </c>
-      <c r="V24">
-        <v>0</v>
-      </c>
-      <c r="W24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23">
+    </row>
+    <row r="25" spans="1:21">
       <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>25</v>
+        <v>0</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -2232,19 +1879,13 @@
       <c r="U25">
         <v>0</v>
       </c>
-      <c r="V25">
-        <v>0</v>
-      </c>
-      <c r="W25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:23">
+    </row>
+    <row r="26" spans="1:21">
       <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>26</v>
+        <v>0</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -2303,19 +1944,13 @@
       <c r="U26">
         <v>0</v>
       </c>
-      <c r="V26">
-        <v>0</v>
-      </c>
-      <c r="W26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:23">
+    </row>
+    <row r="27" spans="1:21">
       <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>27</v>
+        <v>0</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -2374,19 +2009,13 @@
       <c r="U27">
         <v>0</v>
       </c>
-      <c r="V27">
-        <v>0</v>
-      </c>
-      <c r="W27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23">
+    </row>
+    <row r="28" spans="1:21">
       <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="s">
-        <v>28</v>
+        <v>0</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -2445,19 +2074,13 @@
       <c r="U28">
         <v>0</v>
       </c>
-      <c r="V28">
-        <v>0</v>
-      </c>
-      <c r="W28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:23">
+    </row>
+    <row r="29" spans="1:21">
       <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" t="s">
-        <v>29</v>
+        <v>0</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -2516,19 +2139,13 @@
       <c r="U29">
         <v>0</v>
       </c>
-      <c r="V29">
-        <v>0</v>
-      </c>
-      <c r="W29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:23">
+    </row>
+    <row r="30" spans="1:21">
       <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30" t="s">
-        <v>30</v>
+        <v>0</v>
+      </c>
+      <c r="B30">
+        <v>0</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -2587,19 +2204,13 @@
       <c r="U30">
         <v>0</v>
       </c>
-      <c r="V30">
-        <v>0</v>
-      </c>
-      <c r="W30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:23">
+    </row>
+    <row r="31" spans="1:21">
       <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31" t="s">
-        <v>31</v>
+        <v>0</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -2658,19 +2269,13 @@
       <c r="U31">
         <v>0</v>
       </c>
-      <c r="V31">
-        <v>0</v>
-      </c>
-      <c r="W31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:23">
+    </row>
+    <row r="32" spans="1:21">
       <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" t="s">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -2729,19 +2334,13 @@
       <c r="U32">
         <v>0</v>
       </c>
-      <c r="V32">
-        <v>0</v>
-      </c>
-      <c r="W32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:23">
+    </row>
+    <row r="33" spans="1:21">
       <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33" t="s">
-        <v>33</v>
+        <v>0</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -2800,19 +2399,13 @@
       <c r="U33">
         <v>0</v>
       </c>
-      <c r="V33">
-        <v>0</v>
-      </c>
-      <c r="W33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:23">
+    </row>
+    <row r="34" spans="1:21">
       <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34" t="s">
-        <v>34</v>
+        <v>0</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -2871,19 +2464,13 @@
       <c r="U34">
         <v>0</v>
       </c>
-      <c r="V34">
-        <v>0</v>
-      </c>
-      <c r="W34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:23">
+    </row>
+    <row r="35" spans="1:21">
       <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35" t="s">
-        <v>35</v>
+        <v>0</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
       </c>
       <c r="C35">
         <v>0</v>
@@ -2942,19 +2529,13 @@
       <c r="U35">
         <v>0</v>
       </c>
-      <c r="V35">
-        <v>0</v>
-      </c>
-      <c r="W35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:23">
+    </row>
+    <row r="36" spans="1:21">
       <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36" t="s">
-        <v>36</v>
+        <v>0</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -3013,19 +2594,13 @@
       <c r="U36">
         <v>0</v>
       </c>
-      <c r="V36">
-        <v>0</v>
-      </c>
-      <c r="W36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:23">
+    </row>
+    <row r="37" spans="1:21">
       <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37" t="s">
-        <v>37</v>
+        <v>0</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -3084,19 +2659,13 @@
       <c r="U37">
         <v>0</v>
       </c>
-      <c r="V37">
-        <v>0</v>
-      </c>
-      <c r="W37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:23">
+    </row>
+    <row r="38" spans="1:21">
       <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38" t="s">
-        <v>38</v>
+        <v>0</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -3155,19 +2724,13 @@
       <c r="U38">
         <v>0</v>
       </c>
-      <c r="V38">
-        <v>0</v>
-      </c>
-      <c r="W38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:23">
+    </row>
+    <row r="39" spans="1:21">
       <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39" t="s">
-        <v>39</v>
+        <v>0</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -3226,19 +2789,13 @@
       <c r="U39">
         <v>0</v>
       </c>
-      <c r="V39">
-        <v>0</v>
-      </c>
-      <c r="W39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:23">
+    </row>
+    <row r="40" spans="1:21">
       <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40" t="s">
-        <v>40</v>
+        <v>0</v>
+      </c>
+      <c r="B40">
+        <v>0</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -3297,19 +2854,13 @@
       <c r="U40">
         <v>0</v>
       </c>
-      <c r="V40">
-        <v>0</v>
-      </c>
-      <c r="W40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:23">
+    </row>
+    <row r="41" spans="1:21">
       <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" t="s">
-        <v>41</v>
+        <v>0</v>
+      </c>
+      <c r="B41">
+        <v>0</v>
       </c>
       <c r="C41">
         <v>0</v>
@@ -3368,19 +2919,13 @@
       <c r="U41">
         <v>0</v>
       </c>
-      <c r="V41">
-        <v>0</v>
-      </c>
-      <c r="W41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:23">
+    </row>
+    <row r="42" spans="1:21">
       <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42" t="s">
-        <v>42</v>
+        <v>0</v>
+      </c>
+      <c r="B42">
+        <v>0</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -3439,19 +2984,13 @@
       <c r="U42">
         <v>0</v>
       </c>
-      <c r="V42">
-        <v>0</v>
-      </c>
-      <c r="W42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:23">
+    </row>
+    <row r="43" spans="1:21">
       <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43" t="s">
-        <v>43</v>
+        <v>0</v>
+      </c>
+      <c r="B43">
+        <v>0</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -3510,19 +3049,13 @@
       <c r="U43">
         <v>0</v>
       </c>
-      <c r="V43">
-        <v>0</v>
-      </c>
-      <c r="W43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:23">
+    </row>
+    <row r="44" spans="1:21">
       <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44" t="s">
-        <v>44</v>
+        <v>0</v>
+      </c>
+      <c r="B44">
+        <v>0</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -3581,19 +3114,13 @@
       <c r="U44">
         <v>0</v>
       </c>
-      <c r="V44">
-        <v>0</v>
-      </c>
-      <c r="W44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:23">
+    </row>
+    <row r="45" spans="1:21">
       <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45" t="s">
-        <v>45</v>
+        <v>0</v>
+      </c>
+      <c r="B45">
+        <v>0</v>
       </c>
       <c r="C45">
         <v>0</v>
@@ -3652,19 +3179,13 @@
       <c r="U45">
         <v>0</v>
       </c>
-      <c r="V45">
-        <v>0</v>
-      </c>
-      <c r="W45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:23">
+    </row>
+    <row r="46" spans="1:21">
       <c r="A46">
-        <v>45</v>
-      </c>
-      <c r="B46" t="s">
-        <v>46</v>
+        <v>0</v>
+      </c>
+      <c r="B46">
+        <v>0</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -3723,19 +3244,13 @@
       <c r="U46">
         <v>0</v>
       </c>
-      <c r="V46">
-        <v>0</v>
-      </c>
-      <c r="W46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:23">
+    </row>
+    <row r="47" spans="1:21">
       <c r="A47">
-        <v>46</v>
-      </c>
-      <c r="B47" t="s">
-        <v>47</v>
+        <v>0</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
       </c>
       <c r="C47">
         <v>0</v>
@@ -3794,19 +3309,13 @@
       <c r="U47">
         <v>0</v>
       </c>
-      <c r="V47">
-        <v>0</v>
-      </c>
-      <c r="W47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:23">
+    </row>
+    <row r="48" spans="1:21">
       <c r="A48">
-        <v>47</v>
-      </c>
-      <c r="B48" t="s">
-        <v>48</v>
+        <v>0</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
       </c>
       <c r="C48">
         <v>0</v>
@@ -3865,19 +3374,13 @@
       <c r="U48">
         <v>0</v>
       </c>
-      <c r="V48">
-        <v>0</v>
-      </c>
-      <c r="W48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:23">
+    </row>
+    <row r="49" spans="1:21">
       <c r="A49">
-        <v>48</v>
-      </c>
-      <c r="B49" t="s">
-        <v>49</v>
+        <v>0</v>
+      </c>
+      <c r="B49">
+        <v>0</v>
       </c>
       <c r="C49">
         <v>0</v>
@@ -3936,19 +3439,13 @@
       <c r="U49">
         <v>0</v>
       </c>
-      <c r="V49">
-        <v>0</v>
-      </c>
-      <c r="W49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:23">
+    </row>
+    <row r="50" spans="1:21">
       <c r="A50">
-        <v>49</v>
-      </c>
-      <c r="B50" t="s">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="B50">
+        <v>0</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -4007,19 +3504,13 @@
       <c r="U50">
         <v>0</v>
       </c>
-      <c r="V50">
-        <v>0</v>
-      </c>
-      <c r="W50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:23">
+    </row>
+    <row r="51" spans="1:21">
       <c r="A51">
-        <v>50</v>
-      </c>
-      <c r="B51" t="s">
-        <v>51</v>
+        <v>0</v>
+      </c>
+      <c r="B51">
+        <v>0</v>
       </c>
       <c r="C51">
         <v>0</v>
@@ -4078,19 +3569,13 @@
       <c r="U51">
         <v>0</v>
       </c>
-      <c r="V51">
-        <v>0</v>
-      </c>
-      <c r="W51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:23">
+    </row>
+    <row r="52" spans="1:21">
       <c r="A52">
-        <v>51</v>
-      </c>
-      <c r="B52" t="s">
-        <v>52</v>
+        <v>0</v>
+      </c>
+      <c r="B52">
+        <v>0</v>
       </c>
       <c r="C52">
         <v>0</v>
@@ -4149,19 +3634,13 @@
       <c r="U52">
         <v>0</v>
       </c>
-      <c r="V52">
-        <v>0</v>
-      </c>
-      <c r="W52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:23">
+    </row>
+    <row r="53" spans="1:21">
       <c r="A53">
-        <v>52</v>
-      </c>
-      <c r="B53" t="s">
-        <v>53</v>
+        <v>0</v>
+      </c>
+      <c r="B53">
+        <v>0</v>
       </c>
       <c r="C53">
         <v>0</v>
@@ -4220,19 +3699,13 @@
       <c r="U53">
         <v>0</v>
       </c>
-      <c r="V53">
-        <v>0</v>
-      </c>
-      <c r="W53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:23">
+    </row>
+    <row r="54" spans="1:21">
       <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54" t="s">
-        <v>54</v>
+        <v>0</v>
+      </c>
+      <c r="B54">
+        <v>0</v>
       </c>
       <c r="C54">
         <v>0</v>
@@ -4291,19 +3764,13 @@
       <c r="U54">
         <v>0</v>
       </c>
-      <c r="V54">
-        <v>0</v>
-      </c>
-      <c r="W54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:23">
+    </row>
+    <row r="55" spans="1:21">
       <c r="A55">
-        <v>54</v>
-      </c>
-      <c r="B55" t="s">
-        <v>55</v>
+        <v>0</v>
+      </c>
+      <c r="B55">
+        <v>0</v>
       </c>
       <c r="C55">
         <v>0</v>
@@ -4362,19 +3829,13 @@
       <c r="U55">
         <v>0</v>
       </c>
-      <c r="V55">
-        <v>0</v>
-      </c>
-      <c r="W55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:23">
+    </row>
+    <row r="56" spans="1:21">
       <c r="A56">
-        <v>55</v>
-      </c>
-      <c r="B56" t="s">
-        <v>56</v>
+        <v>0</v>
+      </c>
+      <c r="B56">
+        <v>0</v>
       </c>
       <c r="C56">
         <v>0</v>
@@ -4433,19 +3894,13 @@
       <c r="U56">
         <v>0</v>
       </c>
-      <c r="V56">
-        <v>0</v>
-      </c>
-      <c r="W56">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:23">
+    </row>
+    <row r="57" spans="1:21">
       <c r="A57">
-        <v>56</v>
-      </c>
-      <c r="B57" t="s">
-        <v>57</v>
+        <v>0</v>
+      </c>
+      <c r="B57">
+        <v>0</v>
       </c>
       <c r="C57">
         <v>0</v>
@@ -4504,19 +3959,13 @@
       <c r="U57">
         <v>0</v>
       </c>
-      <c r="V57">
-        <v>0</v>
-      </c>
-      <c r="W57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:23">
+    </row>
+    <row r="58" spans="1:21">
       <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58" t="s">
-        <v>58</v>
+        <v>0</v>
+      </c>
+      <c r="B58">
+        <v>0</v>
       </c>
       <c r="C58">
         <v>0</v>
@@ -4575,19 +4024,13 @@
       <c r="U58">
         <v>0</v>
       </c>
-      <c r="V58">
-        <v>0</v>
-      </c>
-      <c r="W58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:23">
+    </row>
+    <row r="59" spans="1:21">
       <c r="A59">
-        <v>58</v>
-      </c>
-      <c r="B59" t="s">
-        <v>59</v>
+        <v>0</v>
+      </c>
+      <c r="B59">
+        <v>0</v>
       </c>
       <c r="C59">
         <v>0</v>
@@ -4646,19 +4089,13 @@
       <c r="U59">
         <v>0</v>
       </c>
-      <c r="V59">
-        <v>0</v>
-      </c>
-      <c r="W59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:23">
+    </row>
+    <row r="60" spans="1:21">
       <c r="A60">
-        <v>59</v>
-      </c>
-      <c r="B60" t="s">
-        <v>60</v>
+        <v>0</v>
+      </c>
+      <c r="B60">
+        <v>0</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -4717,19 +4154,13 @@
       <c r="U60">
         <v>0</v>
       </c>
-      <c r="V60">
-        <v>0</v>
-      </c>
-      <c r="W60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:23">
+    </row>
+    <row r="61" spans="1:21">
       <c r="A61">
-        <v>60</v>
-      </c>
-      <c r="B61" t="s">
-        <v>61</v>
+        <v>0</v>
+      </c>
+      <c r="B61">
+        <v>0</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -4788,19 +4219,13 @@
       <c r="U61">
         <v>0</v>
       </c>
-      <c r="V61">
-        <v>0</v>
-      </c>
-      <c r="W61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:23">
+    </row>
+    <row r="62" spans="1:21">
       <c r="A62">
-        <v>61</v>
-      </c>
-      <c r="B62" t="s">
-        <v>62</v>
+        <v>0</v>
+      </c>
+      <c r="B62">
+        <v>0</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -4859,19 +4284,13 @@
       <c r="U62">
         <v>0</v>
       </c>
-      <c r="V62">
-        <v>0</v>
-      </c>
-      <c r="W62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:23">
+    </row>
+    <row r="63" spans="1:21">
       <c r="A63">
-        <v>62</v>
-      </c>
-      <c r="B63" t="s">
-        <v>63</v>
+        <v>0</v>
+      </c>
+      <c r="B63">
+        <v>0</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -4930,19 +4349,13 @@
       <c r="U63">
         <v>0</v>
       </c>
-      <c r="V63">
-        <v>0</v>
-      </c>
-      <c r="W63">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:23">
+    </row>
+    <row r="64" spans="1:21">
       <c r="A64">
-        <v>63</v>
-      </c>
-      <c r="B64" t="s">
-        <v>64</v>
+        <v>0</v>
+      </c>
+      <c r="B64">
+        <v>0</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -5001,19 +4414,13 @@
       <c r="U64">
         <v>0</v>
       </c>
-      <c r="V64">
-        <v>0</v>
-      </c>
-      <c r="W64">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:23">
+    </row>
+    <row r="65" spans="1:21">
       <c r="A65">
-        <v>64</v>
-      </c>
-      <c r="B65" t="s">
-        <v>65</v>
+        <v>0</v>
+      </c>
+      <c r="B65">
+        <v>0</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -5072,19 +4479,13 @@
       <c r="U65">
         <v>0</v>
       </c>
-      <c r="V65">
-        <v>0</v>
-      </c>
-      <c r="W65">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:23">
+    </row>
+    <row r="66" spans="1:21">
       <c r="A66">
-        <v>65</v>
-      </c>
-      <c r="B66" t="s">
-        <v>66</v>
+        <v>0</v>
+      </c>
+      <c r="B66">
+        <v>0</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -5143,86 +4544,9 @@
       <c r="U66">
         <v>0</v>
       </c>
-      <c r="V66">
-        <v>0</v>
-      </c>
-      <c r="W66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:23">
-      <c r="A67">
-        <v>66</v>
-      </c>
-      <c r="B67" t="s">
-        <v>67</v>
-      </c>
-      <c r="C67">
-        <v>0</v>
-      </c>
-      <c r="D67">
-        <v>0</v>
-      </c>
-      <c r="E67">
-        <v>0</v>
-      </c>
-      <c r="F67">
-        <v>0</v>
-      </c>
-      <c r="G67">
-        <v>0</v>
-      </c>
-      <c r="H67">
-        <v>0</v>
-      </c>
-      <c r="I67">
-        <v>0</v>
-      </c>
-      <c r="J67">
-        <v>0</v>
-      </c>
-      <c r="K67">
-        <v>0</v>
-      </c>
-      <c r="L67">
-        <v>0</v>
-      </c>
-      <c r="M67">
-        <v>0</v>
-      </c>
-      <c r="N67">
-        <v>0</v>
-      </c>
-      <c r="O67">
-        <v>0</v>
-      </c>
-      <c r="P67">
-        <v>0</v>
-      </c>
-      <c r="Q67">
-        <v>0</v>
-      </c>
-      <c r="R67">
-        <v>0</v>
-      </c>
-      <c r="S67">
-        <v>0</v>
-      </c>
-      <c r="T67">
-        <v>0</v>
-      </c>
-      <c r="U67">
-        <v>0</v>
-      </c>
-      <c r="V67">
-        <v>0</v>
-      </c>
-      <c r="W67">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:W67">
+  <conditionalFormatting sqref="A1:U66">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Comparison BAU and LAS
</commit_message>
<xml_diff>
--- a/SType2.xlsx
+++ b/SType2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_LASSO\LAS_Simulation_Jateng\I-O_Analysis\Regional-Economy---Jawa-Tengah\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC004F7D-703C-4BE4-AAA7-0B26F71BC891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AE829C-952D-4970-93DF-BFE0F4362C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E5C01E36-476D-4251-853A-101B82F37DF2}"/>
   </bookViews>
@@ -36,10 +36,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -358,31 +354,31 @@
         <v>0.03</v>
       </c>
       <c r="M2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="N2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="O2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="P2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="Q2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="R2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.2</v>
       </c>
       <c r="S2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.2</v>
       </c>
       <c r="T2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.2</v>
       </c>
       <c r="U2">
-        <v>7.0000000000000007E-2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -423,31 +419,31 @@
         <v>0.03</v>
       </c>
       <c r="M3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="N3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="P3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="Q3">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="R3">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="S3">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="T3">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="U3">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -488,31 +484,31 @@
         <v>0.03</v>
       </c>
       <c r="M4">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="N4">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="O4">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="P4">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="Q4">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="R4">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="S4">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="T4">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="U4">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5" spans="1:21">
@@ -689,25 +685,25 @@
         <v>0.05</v>
       </c>
       <c r="O7">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="P7">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="Q7">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="R7">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="S7">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="T7">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="U7">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8" spans="1:21">
@@ -754,25 +750,25 @@
         <v>0.05</v>
       </c>
       <c r="O8">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="P8">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="Q8">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="R8">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="S8">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="T8">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="U8">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="9" spans="1:21">
@@ -890,19 +886,19 @@
         <v>0.05</v>
       </c>
       <c r="Q10">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="R10">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="S10">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="T10">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="U10">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11" spans="1:21">
@@ -1209,25 +1205,25 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="O15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="P15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="Q15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="R15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="S15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="T15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="U15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="16" spans="1:21">

</xml_diff>

<commit_message>
excercise Stype2 without smoothing
</commit_message>
<xml_diff>
--- a/SType2.xlsx
+++ b/SType2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_LASSO\LAS_Simulation_Jateng\I-O_Analysis\Regional-Economy---Jawa-Tengah\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy---Jawa-Tengah/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC004F7D-703C-4BE4-AAA7-0B26F71BC891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{DC004F7D-703C-4BE4-AAA7-0B26F71BC891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC5312B9-E33D-47D0-BAE4-092318535DB0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E5C01E36-476D-4251-853A-101B82F37DF2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E5C01E36-476D-4251-853A-101B82F37DF2}"/>
   </bookViews>
   <sheets>
     <sheet name="SType2" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -253,7 +249,7 @@
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:U66"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1">
@@ -263,61 +259,61 @@
         <v>0</v>
       </c>
       <c r="C1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="I1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="J1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="K1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="L1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="M1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="N1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="O1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="P1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="Q1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="R1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="S1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="T1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="U1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -396,58 +392,58 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E3">
-        <v>0.01</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="F3">
-        <v>0.01</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="G3">
-        <v>0.01</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="H3">
-        <v>0.01</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="I3">
-        <v>0.03</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="J3">
-        <v>0.03</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="K3">
-        <v>0.03</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="L3">
-        <v>0.03</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="M3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="N3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="P3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="Q3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="R3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="S3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="T3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="U3">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -458,61 +454,61 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="E4">
-        <v>0.01</v>
+        <v>0.09</v>
       </c>
       <c r="F4">
-        <v>0.01</v>
+        <v>0.09</v>
       </c>
       <c r="G4">
-        <v>0.01</v>
+        <v>0.09</v>
       </c>
       <c r="H4">
-        <v>0.01</v>
+        <v>0.09</v>
       </c>
       <c r="I4">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
       <c r="J4">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
       <c r="K4">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
       <c r="L4">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
       <c r="M4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="N4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="O4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="P4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="Q4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="R4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="S4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="T4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="U4">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="5" spans="1:21">
@@ -523,61 +519,61 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="Q5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="T5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="U5">
-        <v>0</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="6" spans="1:21">
@@ -659,55 +655,55 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>0.03</v>
+        <v>0.16</v>
       </c>
       <c r="J7">
-        <v>0.03</v>
+        <v>0.16</v>
       </c>
       <c r="K7">
-        <v>0.03</v>
+        <v>0.16</v>
       </c>
       <c r="L7">
-        <v>0.03</v>
+        <v>0.16</v>
       </c>
       <c r="M7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="N7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="O7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="P7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="Q7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="R7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="S7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="T7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="U7">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="8" spans="1:21">
@@ -724,55 +720,55 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>0.01</v>
+        <v>0.51</v>
       </c>
       <c r="F8">
-        <v>0.01</v>
+        <v>0.51</v>
       </c>
       <c r="G8">
-        <v>0.01</v>
+        <v>0.51</v>
       </c>
       <c r="H8">
-        <v>0.01</v>
+        <v>0.51</v>
       </c>
       <c r="I8">
-        <v>0.03</v>
+        <v>0.51</v>
       </c>
       <c r="J8">
-        <v>0.03</v>
+        <v>0.51</v>
       </c>
       <c r="K8">
-        <v>0.03</v>
+        <v>0.51</v>
       </c>
       <c r="L8">
-        <v>0.03</v>
+        <v>0.51</v>
       </c>
       <c r="M8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
       <c r="N8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
       <c r="O8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
       <c r="P8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
       <c r="Q8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
       <c r="R8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
       <c r="S8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
       <c r="T8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
       <c r="U8">
-        <v>0.05</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="9" spans="1:21">
@@ -1070,34 +1066,34 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="M13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="N13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="O13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="P13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="Q13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="S13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="T13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="U13">
-        <v>0</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="14" spans="1:21">
@@ -1176,58 +1172,58 @@
         <v>0</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="E15">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="F15">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="G15">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="H15">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="I15">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="J15">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="K15">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="L15">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="M15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="N15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="O15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="P15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="Q15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="R15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="S15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="T15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="U15">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="16" spans="1:21">

</xml_diff>